<commit_message>
upd mpi - get rid of send/recv
</commit_message>
<xml_diff>
--- a/reports/lab3/chart.xlsx
+++ b/reports/lab3/chart.xlsx
@@ -98,6 +98,7 @@
     </font>
     <font>
       <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -828,22 +829,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.666</c:v>
+                  <c:v>0.088</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.886</c:v>
+                  <c:v>0.416</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.901</c:v>
+                  <c:v>1.044</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>29.287</c:v>
+                  <c:v>4.408</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>63.102</c:v>
+                  <c:v>9.297</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>311.401</c:v>
+                  <c:v>43.856</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -956,22 +957,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.888</c:v>
+                  <c:v>0.069</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.103</c:v>
+                  <c:v>0.348</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.295</c:v>
+                  <c:v>0.622</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>21.448</c:v>
+                  <c:v>3.165</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>42.692</c:v>
+                  <c:v>6.214</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>211.916</c:v>
+                  <c:v>38.22</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1019,12 +1020,16 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" strike="noStrike" u="none">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1080,22 +1085,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.291</c:v>
+                  <c:v>0.069</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.422</c:v>
+                  <c:v>0.348</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.224</c:v>
+                  <c:v>0.622</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>16.039</c:v>
+                  <c:v>3.165</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>32.03</c:v>
+                  <c:v>6.214</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>166.743</c:v>
+                  <c:v>38.22</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1110,11 +1115,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="73840808"/>
-        <c:axId val="83102908"/>
+        <c:axId val="96498584"/>
+        <c:axId val="15403592"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="73840808"/>
+        <c:axId val="96498584"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1134,6 +1139,9 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr b="0" sz="900" strike="noStrike" u="none">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
@@ -1176,7 +1184,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83102908"/>
+        <c:crossAx val="15403592"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1184,7 +1192,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="83102908"/>
+        <c:axId val="15403592"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1213,6 +1221,9 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr b="0" sz="900" strike="noStrike" u="none">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:rPr>
@@ -1255,7 +1266,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73840808"/>
+        <c:crossAx val="96498584"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1318,9 +1329,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>694080</xdr:colOff>
+      <xdr:colOff>693720</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>179280</xdr:rowOff>
+      <xdr:rowOff>178920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1329,7 +1340,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="523440" y="1769760"/>
-        <a:ext cx="8434440" cy="4743720"/>
+        <a:ext cx="8434080" cy="4743360"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1579,13 +1590,13 @@
         <v>1.076</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.666</v>
+        <v>0.088</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>0.888</v>
+        <v>0.069</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>0.291</v>
+        <v>0.069</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1602,13 +1613,13 @@
         <v>5.721</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>2.886</v>
+        <v>0.416</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>2.103</v>
+        <v>0.348</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>2.422</v>
+        <v>0.348</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1625,13 +1636,13 @@
         <v>11.789</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>5.901</v>
+        <v>1.044</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>4.295</v>
+        <v>0.622</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>3.224</v>
+        <v>0.622</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1648,13 +1659,13 @@
         <v>59.529</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>29.287</v>
+        <v>4.408</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>21.448</v>
+        <v>3.165</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>16.039</v>
+        <v>3.165</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1671,13 +1682,13 @@
         <v>118.678</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>63.102</v>
+        <v>9.297</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>42.692</v>
+        <v>6.214</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>32.03</v>
+        <v>6.214</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1694,13 +1705,13 @@
         <v>579.842</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>311.401</v>
+        <v>43.856</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>211.916</v>
+        <v>38.22</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>166.743</v>
+        <v>38.22</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>